<commit_message>
Upload RALVEN 5.2 reviewed recovery model and template
Post-submission update: explicit cash-funded operating recovery, annual paths and financing obligations, coordinated scenario/simulation/Excel/PDF funding gates, and EV/Sales cross-check. 144 tests and seven independent spreadsheet cases pass. Preserve archived BMRI results and submission baseline; remaining source and sector-model work is documented.
</commit_message>
<xml_diff>
--- a/RALVEN_Input_Template.xlsx
+++ b/RALVEN_Input_Template.xlsx
@@ -2,11 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" r:id="R5cd088e52698431e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inputs" sheetId="2" r:id="R9c4ce899c22f413a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="3" r:id="Reea662bb700148b2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Historical" sheetId="4" r:id="Rc8d3dd4d28994d48"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Peers" sheetId="5" r:id="R75889266a3de4043"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" r:id="R51bfa5220dd24afe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inputs" sheetId="2" r:id="R9f6204f3ada148f2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="3" r:id="R993d6978ba2e4b78"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Historical" sheetId="4" r:id="R2140e2ec1231464c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Peers" sheetId="5" r:id="R546ba3a09c38467e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recovery Inputs" sheetId="6" r:id="R9e59c8ab77cd472d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Driver Paths" sheetId="7" r:id="R22487a1080914256"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -17,11 +19,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="2">
-    <x:numFmt numFmtId="200" formatCode="#,##0.00;(#,##0.00);&quot;-&quot;"/>
-    <x:numFmt numFmtId="201" formatCode="@"/>
+  <x:numFmts count="3">
+    <x:numFmt numFmtId="200" formatCode="@"/>
+    <x:numFmt numFmtId="201" formatCode="0.0%"/>
+    <x:numFmt numFmtId="202" formatCode="0.00"/>
   </x:numFmts>
-  <x:fonts count="4">
+  <x:fonts count="5">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -40,6 +43,11 @@
     <x:font>
       <x:sz val="10"/>
       <x:color rgb="FF1A5BBD"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF21784F"/>
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
@@ -73,16 +81,42 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="9">
+  <x:cellXfs count="13">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="200" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="200" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="200" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="201" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="201" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="200" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="200" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -286,16 +320,16 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="40" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="23" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="95" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="23" customHeight="1">
+    <x:row r="1" ht="24" customHeight="1">
       <x:c r="A1" s="5" t="str">
         <x:v>RALVEN / INPUT TEMPLATE</x:v>
       </x:c>
       <x:c r="B1" s="4"/>
     </x:row>
-    <x:row r="2" ht="23" customHeight="1">
+    <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="6" t="str">
         <x:v>Workflow</x:v>
       </x:c>
@@ -303,7 +337,7 @@
         <x:v>Replace sample data with verified annual IDR data, then upload this .xlsx.</x:v>
       </x:c>
     </x:row>
-    <x:row r="3" ht="23" customHeight="1">
+    <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="6" t="str">
         <x:v>Units</x:v>
       </x:c>
@@ -311,7 +345,7 @@
         <x:v>Financial amounts in IDR billions. Shares in billions. Price in IDR per share.</x:v>
       </x:c>
     </x:row>
-    <x:row r="4" ht="23" customHeight="1">
+    <x:row r="4" ht="35" customHeight="1">
       <x:c r="A4" s="6" t="str">
         <x:v>Source</x:v>
       </x:c>
@@ -319,7 +353,7 @@
         <x:v>Give the issuer report URL, reporting period, quote source, and publication date in Inputs.source.</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="23" customHeight="1">
+    <x:row r="5" ht="35" customHeight="1">
       <x:c r="A5" s="6" t="str">
         <x:v>Missing values</x:v>
       </x:c>
@@ -327,7 +361,7 @@
         <x:v>Do not replace missing data with zero. Use zero only after verifying absence of that item.</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="23" customHeight="1">
+    <x:row r="6" ht="35" customHeight="1">
       <x:c r="A6" s="6" t="str">
         <x:v>Historical</x:v>
       </x:c>
@@ -335,7 +369,7 @@
         <x:v>Label each historical period ANNUAL or TTM with its actual end date. Use matching fiscal periods. No automatic quarterly annualization.</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="23" customHeight="1">
+    <x:row r="7" ht="35" customHeight="1">
       <x:c r="A7" s="6" t="str">
         <x:v>Peers</x:v>
       </x:c>
@@ -343,7 +377,7 @@
         <x:v>At least 3 eligible peers per multiple. Same industry/currency. Annual or TTM end dates within 100 days; quotes at most 7 days old. Peer metadata is retained at export.</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="23" customHeight="1">
+    <x:row r="8" ht="35" customHeight="1">
       <x:c r="A8" s="6" t="str">
         <x:v>Capital</x:v>
       </x:c>
@@ -351,7 +385,7 @@
         <x:v>Debt includes interest-bearing leases. Cash must exclude restricted cash. Minority and preferred are claim values.</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="23" customHeight="1">
+    <x:row r="9" ht="24" customHeight="1">
       <x:c r="A9" s="6" t="str">
         <x:v>Financial firms</x:v>
       </x:c>
@@ -359,7 +393,7 @@
         <x:v>Debt and cash are excluded from enterprise bridges. Use DDM, P/E and P/B.</x:v>
       </x:c>
     </x:row>
-    <x:row r="10" ht="23" customHeight="1">
+    <x:row r="10" ht="24" customHeight="1">
       <x:c r="A10" s="6" t="str">
         <x:v>Assumptions</x:v>
       </x:c>
@@ -367,7 +401,7 @@
         <x:v>Rates are decimals: 0.06 = 6%. These are analyst assumptions, not provider forecasts.</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="23" customHeight="1">
+    <x:row r="11" ht="35" customHeight="1">
       <x:c r="A11" s="6" t="str">
         <x:v>Sample status</x:v>
       </x:c>
@@ -375,7 +409,7 @@
         <x:v>mode must remain demo for sample data. Set mode to import only after entering verified values.</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" ht="23" customHeight="1">
+    <x:row r="12" ht="35" customHeight="1">
       <x:c r="A12" s="6" t="str">
         <x:v>Security</x:v>
       </x:c>
@@ -393,16 +427,16 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="40" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="23" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="95" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="23" customHeight="1">
+    <x:row r="1" ht="24" customHeight="1">
       <x:c r="A1" s="5" t="str">
         <x:v>RALVEN / DATA INPUTS</x:v>
       </x:c>
       <x:c r="B1" s="4"/>
     </x:row>
-    <x:row r="2" ht="23" customHeight="1">
+    <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="6" t="str">
         <x:v>Field</x:v>
       </x:c>
@@ -410,7 +444,7 @@
         <x:v>Value</x:v>
       </x:c>
     </x:row>
-    <x:row r="3" ht="23" customHeight="1">
+    <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="6" t="str">
         <x:v>ticker</x:v>
       </x:c>
@@ -418,7 +452,7 @@
         <x:v>TLKM</x:v>
       </x:c>
     </x:row>
-    <x:row r="4" ht="23" customHeight="1">
+    <x:row r="4" ht="24" customHeight="1">
       <x:c r="A4" s="6" t="str">
         <x:v>name</x:v>
       </x:c>
@@ -426,7 +460,7 @@
         <x:v>Telkom Indonesia (Persero) Tbk</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="23" customHeight="1">
+    <x:row r="5" ht="24" customHeight="1">
       <x:c r="A5" s="6" t="str">
         <x:v>sector</x:v>
       </x:c>
@@ -434,7 +468,7 @@
         <x:v>Communication Services</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="23" customHeight="1">
+    <x:row r="6" ht="24" customHeight="1">
       <x:c r="A6" s="6" t="str">
         <x:v>currency</x:v>
       </x:c>
@@ -442,7 +476,7 @@
         <x:v>IDR</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="23" customHeight="1">
+    <x:row r="7" ht="24" customHeight="1">
       <x:c r="A7" s="6" t="str">
         <x:v>units</x:v>
       </x:c>
@@ -450,7 +484,7 @@
         <x:v>IDR bn / shares bn</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="23" customHeight="1">
+    <x:row r="8" ht="24" customHeight="1">
       <x:c r="A8" s="6" t="str">
         <x:v>period</x:v>
       </x:c>
@@ -458,7 +492,7 @@
         <x:v>2025-12-31</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="23" customHeight="1">
+    <x:row r="9" ht="24" customHeight="1">
       <x:c r="A9" s="6" t="str">
         <x:v>priceDate</x:v>
       </x:c>
@@ -466,7 +500,7 @@
         <x:v>2026-10-23</x:v>
       </x:c>
     </x:row>
-    <x:row r="10" ht="23" customHeight="1">
+    <x:row r="10" ht="24" customHeight="1">
       <x:c r="A10" s="6" t="str">
         <x:v>valuationDate</x:v>
       </x:c>
@@ -474,7 +508,7 @@
         <x:v>2026-10-24</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="23" customHeight="1">
+    <x:row r="11" ht="24" customHeight="1">
       <x:c r="A11" s="6" t="str">
         <x:v>price</x:v>
       </x:c>
@@ -482,7 +516,7 @@
         <x:v>2750</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" ht="23" customHeight="1">
+    <x:row r="12" ht="24" customHeight="1">
       <x:c r="A12" s="6" t="str">
         <x:v>shares</x:v>
       </x:c>
@@ -490,7 +524,7 @@
         <x:v>99.06</x:v>
       </x:c>
     </x:row>
-    <x:row r="13" ht="23" customHeight="1">
+    <x:row r="13" ht="24" customHeight="1">
       <x:c r="A13" s="6" t="str">
         <x:v>revenue</x:v>
       </x:c>
@@ -498,7 +532,7 @@
         <x:v>150000</x:v>
       </x:c>
     </x:row>
-    <x:row r="14" ht="23" customHeight="1">
+    <x:row r="14" ht="24" customHeight="1">
       <x:c r="A14" s="6" t="str">
         <x:v>ebit</x:v>
       </x:c>
@@ -506,7 +540,7 @@
         <x:v>38800</x:v>
       </x:c>
     </x:row>
-    <x:row r="15" ht="23" customHeight="1">
+    <x:row r="15" ht="24" customHeight="1">
       <x:c r="A15" s="6" t="str">
         <x:v>netIncome</x:v>
       </x:c>
@@ -514,7 +548,7 @@
         <x:v>24500</x:v>
       </x:c>
     </x:row>
-    <x:row r="16" ht="23" customHeight="1">
+    <x:row r="16" ht="24" customHeight="1">
       <x:c r="A16" s="6" t="str">
         <x:v>ebitda</x:v>
       </x:c>
@@ -522,7 +556,7 @@
         <x:v>68000</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="23" customHeight="1">
+    <x:row r="17" ht="24" customHeight="1">
       <x:c r="A17" s="6" t="str">
         <x:v>bookEquity</x:v>
       </x:c>
@@ -530,7 +564,7 @@
         <x:v>134000</x:v>
       </x:c>
     </x:row>
-    <x:row r="18" ht="23" customHeight="1">
+    <x:row r="18" ht="24" customHeight="1">
       <x:c r="A18" s="6" t="str">
         <x:v>debt</x:v>
       </x:c>
@@ -538,7 +572,7 @@
         <x:v>39000</x:v>
       </x:c>
     </x:row>
-    <x:row r="19" ht="23" customHeight="1">
+    <x:row r="19" ht="24" customHeight="1">
       <x:c r="A19" s="6" t="str">
         <x:v>cash</x:v>
       </x:c>
@@ -546,7 +580,7 @@
         <x:v>26000</x:v>
       </x:c>
     </x:row>
-    <x:row r="20" ht="23" customHeight="1">
+    <x:row r="20" ht="24" customHeight="1">
       <x:c r="A20" s="6" t="str">
         <x:v>minority</x:v>
       </x:c>
@@ -554,7 +588,7 @@
         <x:v>1800</x:v>
       </x:c>
     </x:row>
-    <x:row r="21" ht="23" customHeight="1">
+    <x:row r="21" ht="24" customHeight="1">
       <x:c r="A21" s="6" t="str">
         <x:v>preferred</x:v>
       </x:c>
@@ -562,7 +596,7 @@
         <x:v>0</x:v>
       </x:c>
     </x:row>
-    <x:row r="22" ht="23" customHeight="1">
+    <x:row r="22" ht="35" customHeight="1">
       <x:c r="A22" s="6" t="str">
         <x:v>source</x:v>
       </x:c>
@@ -570,7 +604,7 @@
         <x:v>RALVEN synthetic teaching dataset. All amounts, dates and price histories are illustrative, not verified issuer results.</x:v>
       </x:c>
     </x:row>
-    <x:row r="23" ht="23" customHeight="1">
+    <x:row r="23" ht="24" customHeight="1">
       <x:c r="A23" s="6" t="str">
         <x:v>updatedAt</x:v>
       </x:c>
@@ -578,7 +612,7 @@
         <x:v>2026-10-23T17:00:00.000Z</x:v>
       </x:c>
     </x:row>
-    <x:row r="24" ht="23" customHeight="1">
+    <x:row r="24" ht="24" customHeight="1">
       <x:c r="A24" s="6" t="str">
         <x:v>mode</x:v>
       </x:c>
@@ -599,13 +633,13 @@
     <x:col min="2" max="2" width="23" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="23" customHeight="1">
+    <x:row r="1" ht="24" customHeight="1">
       <x:c r="A1" s="5" t="str">
         <x:v>RALVEN / ASSUMPTIONS</x:v>
       </x:c>
       <x:c r="B1" s="4"/>
     </x:row>
-    <x:row r="2" ht="23" customHeight="1">
+    <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="6" t="str">
         <x:v>Parameter</x:v>
       </x:c>
@@ -613,131 +647,131 @@
         <x:v>Value</x:v>
       </x:c>
     </x:row>
-    <x:row r="3" ht="23" customHeight="1">
+    <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="6" t="str">
         <x:v>growth</x:v>
       </x:c>
-      <x:c r="B3" s="8" t="n">
+      <x:c r="B3" s="9" t="n">
         <x:v>0.06</x:v>
       </x:c>
     </x:row>
-    <x:row r="4" ht="23" customHeight="1">
+    <x:row r="4" ht="24" customHeight="1">
       <x:c r="A4" s="6" t="str">
         <x:v>margin</x:v>
       </x:c>
-      <x:c r="B4" s="8" t="n">
+      <x:c r="B4" s="9" t="n">
         <x:v>0.25866666666666666</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="23" customHeight="1">
+    <x:row r="5" ht="24" customHeight="1">
       <x:c r="A5" s="6" t="str">
         <x:v>tax</x:v>
       </x:c>
-      <x:c r="B5" s="8" t="n">
+      <x:c r="B5" s="9" t="n">
         <x:v>0.22</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="23" customHeight="1">
+    <x:row r="6" ht="24" customHeight="1">
       <x:c r="A6" s="6" t="str">
         <x:v>da</x:v>
       </x:c>
-      <x:c r="B6" s="8" t="n">
+      <x:c r="B6" s="9" t="n">
         <x:v>0.19466666666666665</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="23" customHeight="1">
+    <x:row r="7" ht="24" customHeight="1">
       <x:c r="A7" s="6" t="str">
         <x:v>capex</x:v>
       </x:c>
-      <x:c r="B7" s="8" t="n">
+      <x:c r="B7" s="9" t="n">
         <x:v>0.055</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="23" customHeight="1">
+    <x:row r="8" ht="24" customHeight="1">
       <x:c r="A8" s="6" t="str">
         <x:v>nwc</x:v>
       </x:c>
-      <x:c r="B8" s="8" t="n">
+      <x:c r="B8" s="9" t="n">
         <x:v>0.04</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="23" customHeight="1">
+    <x:row r="9" ht="24" customHeight="1">
       <x:c r="A9" s="6" t="str">
         <x:v>rf</x:v>
       </x:c>
-      <x:c r="B9" s="8" t="n">
+      <x:c r="B9" s="9" t="n">
         <x:v>0.065</x:v>
       </x:c>
     </x:row>
-    <x:row r="10" ht="23" customHeight="1">
+    <x:row r="10" ht="24" customHeight="1">
       <x:c r="A10" s="6" t="str">
         <x:v>beta</x:v>
       </x:c>
-      <x:c r="B10" s="8" t="n">
+      <x:c r="B10" s="10" t="n">
         <x:v>0.9</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="23" customHeight="1">
+    <x:row r="11" ht="24" customHeight="1">
       <x:c r="A11" s="6" t="str">
         <x:v>erp</x:v>
       </x:c>
-      <x:c r="B11" s="8" t="n">
+      <x:c r="B11" s="9" t="n">
         <x:v>0.065</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" ht="23" customHeight="1">
+    <x:row r="12" ht="24" customHeight="1">
       <x:c r="A12" s="6" t="str">
         <x:v>kd</x:v>
       </x:c>
-      <x:c r="B12" s="8" t="n">
+      <x:c r="B12" s="9" t="n">
         <x:v>0.085</x:v>
       </x:c>
     </x:row>
-    <x:row r="13" ht="23" customHeight="1">
+    <x:row r="13" ht="24" customHeight="1">
       <x:c r="A13" s="6" t="str">
         <x:v>g</x:v>
       </x:c>
-      <x:c r="B13" s="8" t="n">
+      <x:c r="B13" s="9" t="n">
         <x:v>0.035</x:v>
       </x:c>
     </x:row>
-    <x:row r="14" ht="23" customHeight="1">
+    <x:row r="14" ht="24" customHeight="1">
       <x:c r="A14" s="6" t="str">
         <x:v>roic</x:v>
       </x:c>
-      <x:c r="B14" s="8" t="n">
+      <x:c r="B14" s="9" t="n">
         <x:v>0.14</x:v>
       </x:c>
     </x:row>
-    <x:row r="15" ht="23" customHeight="1">
+    <x:row r="15" ht="24" customHeight="1">
       <x:c r="A15" s="6" t="str">
         <x:v>payout</x:v>
       </x:c>
-      <x:c r="B15" s="8" t="n">
+      <x:c r="B15" s="9" t="n">
         <x:v>0.65</x:v>
       </x:c>
     </x:row>
-    <x:row r="16" ht="23" customHeight="1">
+    <x:row r="16" ht="24" customHeight="1">
       <x:c r="A16" s="6" t="str">
         <x:v>terminalRoe</x:v>
       </x:c>
-      <x:c r="B16" s="8" t="n">
+      <x:c r="B16" s="9" t="n">
         <x:v>0.16</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="23" customHeight="1">
+    <x:row r="17" ht="24" customHeight="1">
       <x:c r="A17" s="6" t="str">
         <x:v>buy</x:v>
       </x:c>
-      <x:c r="B17" s="8" t="n">
+      <x:c r="B17" s="9" t="n">
         <x:v>0.15</x:v>
       </x:c>
     </x:row>
-    <x:row r="18" ht="23" customHeight="1">
+    <x:row r="18" ht="24" customHeight="1">
       <x:c r="A18" s="6" t="str">
         <x:v>sell</x:v>
       </x:c>
-      <x:c r="B18" s="8" t="n">
+      <x:c r="B18" s="9" t="n">
         <x:v>-0.15</x:v>
       </x:c>
     </x:row>
@@ -759,7 +793,7 @@
     <x:col min="7" max="7" width="23" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="23" customHeight="1">
+    <x:row r="1" ht="24" customHeight="1">
       <x:c r="A1" s="5" t="str">
         <x:v>year</x:v>
       </x:c>
@@ -782,8 +816,8 @@
         <x:v>ocf</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="23" customHeight="1">
-      <x:c r="A2" s="2" t="n">
+    <x:row r="2" ht="24" customHeight="1">
+      <x:c r="A2" s="8" t="n">
         <x:v>2023</x:v>
       </x:c>
       <x:c r="B2" s="6" t="str">
@@ -792,21 +826,21 @@
       <x:c r="C2" s="6" t="str">
         <x:v>ANNUAL</x:v>
       </x:c>
-      <x:c r="D2" s="2" t="n">
+      <x:c r="D2" s="8" t="n">
         <x:v>132000</x:v>
       </x:c>
-      <x:c r="E2" s="2" t="n">
+      <x:c r="E2" s="8" t="n">
         <x:v>32592</x:v>
       </x:c>
-      <x:c r="F2" s="2" t="n">
+      <x:c r="F2" s="8" t="n">
         <x:v>19600</x:v>
       </x:c>
-      <x:c r="G2" s="2" t="n">
+      <x:c r="G2" s="8" t="n">
         <x:v>56440</x:v>
       </x:c>
     </x:row>
-    <x:row r="3" ht="23" customHeight="1">
-      <x:c r="A3" s="2" t="n">
+    <x:row r="3" ht="24" customHeight="1">
+      <x:c r="A3" s="8" t="n">
         <x:v>2024</x:v>
       </x:c>
       <x:c r="B3" s="6" t="str">
@@ -815,21 +849,21 @@
       <x:c r="C3" s="6" t="str">
         <x:v>ANNUAL</x:v>
       </x:c>
-      <x:c r="D3" s="2" t="n">
+      <x:c r="D3" s="8" t="n">
         <x:v>141000</x:v>
       </x:c>
-      <x:c r="E3" s="2" t="n">
+      <x:c r="E3" s="8" t="n">
         <x:v>35696</x:v>
       </x:c>
-      <x:c r="F3" s="2" t="n">
+      <x:c r="F3" s="8" t="n">
         <x:v>22050</x:v>
       </x:c>
-      <x:c r="G3" s="2" t="n">
+      <x:c r="G3" s="8" t="n">
         <x:v>61199.99999999999</x:v>
       </x:c>
     </x:row>
-    <x:row r="4" ht="23" customHeight="1">
-      <x:c r="A4" s="2" t="n">
+    <x:row r="4" ht="24" customHeight="1">
+      <x:c r="A4" s="8" t="n">
         <x:v>2025</x:v>
       </x:c>
       <x:c r="B4" s="6" t="str">
@@ -838,16 +872,16 @@
       <x:c r="C4" s="6" t="str">
         <x:v>ANNUAL</x:v>
       </x:c>
-      <x:c r="D4" s="2" t="n">
+      <x:c r="D4" s="8" t="n">
         <x:v>150000</x:v>
       </x:c>
-      <x:c r="E4" s="2" t="n">
+      <x:c r="E4" s="8" t="n">
         <x:v>38800</x:v>
       </x:c>
-      <x:c r="F4" s="2" t="n">
+      <x:c r="F4" s="8" t="n">
         <x:v>24500</x:v>
       </x:c>
-      <x:c r="G4" s="2" t="n">
+      <x:c r="G4" s="8" t="n">
         <x:v>65960</x:v>
       </x:c>
     </x:row>
@@ -882,7 +916,7 @@
     <x:col min="20" max="20" width="23" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="23" customHeight="1">
+    <x:row r="1" ht="24" customHeight="1">
       <x:c r="A1" s="5" t="str">
         <x:v>ticker</x:v>
       </x:c>
@@ -944,7 +978,7 @@
         <x:v>revenue</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="23" customHeight="1">
+    <x:row r="2" ht="24" customHeight="1">
       <x:c r="A2" s="6" t="str">
         <x:v>ISAT</x:v>
       </x:c>
@@ -996,7 +1030,7 @@
       <x:c r="S2" s="2"/>
       <x:c r="T2" s="2"/>
     </x:row>
-    <x:row r="3" ht="23" customHeight="1">
+    <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="6" t="str">
         <x:v>EXCL</x:v>
       </x:c>
@@ -1048,7 +1082,7 @@
       <x:c r="S3" s="2"/>
       <x:c r="T3" s="2"/>
     </x:row>
-    <x:row r="4" ht="23" customHeight="1">
+    <x:row r="4" ht="24" customHeight="1">
       <x:c r="A4" s="6" t="str">
         <x:v>MTEL</x:v>
       </x:c>
@@ -1100,7 +1134,7 @@
       <x:c r="S4" s="2"/>
       <x:c r="T4" s="2"/>
     </x:row>
-    <x:row r="5" ht="23" customHeight="1">
+    <x:row r="5" ht="24" customHeight="1">
       <x:c r="A5" s="6" t="str">
         <x:v>TOWR</x:v>
       </x:c>
@@ -1155,4 +1189,638 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="40" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="95" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="23" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="23" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="23" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="23" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="24" customHeight="1">
+      <x:c r="A1" s="5" t="str">
+        <x:v>CASH-FUNDED RECOVERY / IDR BN</x:v>
+      </x:c>
+      <x:c r="B1" s="4"/>
+      <x:c r="C1" s="4"/>
+      <x:c r="D1" s="4"/>
+      <x:c r="E1" s="4"/>
+      <x:c r="F1" s="4"/>
+    </x:row>
+    <x:row r="2" ht="24" customHeight="1">
+      <x:c r="A2" s="6" t="str">
+        <x:v>Analyst review confirmed</x:v>
+      </x:c>
+      <x:c r="B2" s="8" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C2" s="2"/>
+      <x:c r="D2" s="2"/>
+      <x:c r="E2" s="2"/>
+      <x:c r="F2" s="2"/>
+    </x:row>
+    <x:row r="3" ht="24" customHeight="1">
+      <x:c r="A3" s="6" t="str">
+        <x:v>No new borrowing or equity</x:v>
+      </x:c>
+      <x:c r="B3" s="8" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C3" s="2"/>
+      <x:c r="D3" s="2"/>
+      <x:c r="E3" s="2"/>
+      <x:c r="F3" s="2"/>
+    </x:row>
+    <x:row r="4" ht="24" customHeight="1">
+      <x:c r="A4" s="6" t="str">
+        <x:v>Source URL</x:v>
+      </x:c>
+      <x:c r="B4" s="6" t="str"/>
+      <x:c r="C4" s="2"/>
+      <x:c r="D4" s="2"/>
+      <x:c r="E4" s="2"/>
+      <x:c r="F4" s="2"/>
+    </x:row>
+    <x:row r="5" ht="24" customHeight="1">
+      <x:c r="A5" s="6" t="str">
+        <x:v>Review rationale</x:v>
+      </x:c>
+      <x:c r="B5" s="6" t="str"/>
+      <x:c r="C5" s="2"/>
+      <x:c r="D5" s="2"/>
+      <x:c r="E5" s="2"/>
+      <x:c r="F5" s="2"/>
+    </x:row>
+    <x:row r="6" ht="24" customHeight="1">
+      <x:c r="A6" s="6" t="str">
+        <x:v>Source period</x:v>
+      </x:c>
+      <x:c r="B6" s="6" t="str">
+        <x:v>2025-12-31</x:v>
+      </x:c>
+      <x:c r="C6" s="2"/>
+      <x:c r="D6" s="2"/>
+      <x:c r="E6" s="2"/>
+      <x:c r="F6" s="2"/>
+    </x:row>
+    <x:row r="7" ht="24" customHeight="1">
+      <x:c r="A7" s="6" t="str">
+        <x:v>Review date</x:v>
+      </x:c>
+      <x:c r="B7" s="6" t="str"/>
+      <x:c r="C7" s="2"/>
+      <x:c r="D7" s="2"/>
+      <x:c r="E7" s="2"/>
+      <x:c r="F7" s="2"/>
+    </x:row>
+    <x:row r="8" ht="24" customHeight="1">
+      <x:c r="A8" s="6" t="str">
+        <x:v>Unrestricted available cash</x:v>
+      </x:c>
+      <x:c r="B8" s="2"/>
+      <x:c r="C8" s="2"/>
+      <x:c r="D8" s="2"/>
+      <x:c r="E8" s="2"/>
+      <x:c r="F8" s="2"/>
+    </x:row>
+    <x:row r="9" ht="24" customHeight="1">
+      <x:c r="A9" s="6" t="str">
+        <x:v>Minimum cash reserve</x:v>
+      </x:c>
+      <x:c r="B9" s="2"/>
+      <x:c r="C9" s="2"/>
+      <x:c r="D9" s="2"/>
+      <x:c r="E9" s="2"/>
+      <x:c r="F9" s="2"/>
+    </x:row>
+    <x:row r="10" ht="24" customHeight="1">
+      <x:c r="A10" s="6" t="str">
+        <x:v>Year</x:v>
+      </x:c>
+      <x:c r="B10" s="6" t="str">
+        <x:v>Y1</x:v>
+      </x:c>
+      <x:c r="C10" s="6" t="str">
+        <x:v>Y2</x:v>
+      </x:c>
+      <x:c r="D10" s="6" t="str">
+        <x:v>Y3</x:v>
+      </x:c>
+      <x:c r="E10" s="6" t="str">
+        <x:v>Y4</x:v>
+      </x:c>
+      <x:c r="F10" s="6" t="str">
+        <x:v>Y5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="24" customHeight="1">
+      <x:c r="A11" s="6" t="str">
+        <x:v>After-tax interest</x:v>
+      </x:c>
+      <x:c r="B11" s="2"/>
+      <x:c r="C11" s="2"/>
+      <x:c r="D11" s="2"/>
+      <x:c r="E11" s="2"/>
+      <x:c r="F11" s="2"/>
+    </x:row>
+    <x:row r="12" ht="24" customHeight="1">
+      <x:c r="A12" s="6" t="str">
+        <x:v>Principal cash payments</x:v>
+      </x:c>
+      <x:c r="B12" s="2"/>
+      <x:c r="C12" s="2"/>
+      <x:c r="D12" s="2"/>
+      <x:c r="E12" s="2"/>
+      <x:c r="F12" s="2"/>
+    </x:row>
+    <x:row r="13" ht="24" customHeight="1">
+      <x:c r="A13" s="6" t="str">
+        <x:v>Other cash obligations</x:v>
+      </x:c>
+      <x:c r="B13" s="2"/>
+      <x:c r="C13" s="2"/>
+      <x:c r="D13" s="2"/>
+      <x:c r="E13" s="2"/>
+      <x:c r="F13" s="2"/>
+    </x:row>
+    <x:row r="14" ht="24" customHeight="1">
+      <x:c r="A14" s="6" t="str">
+        <x:v>Valuation date</x:v>
+      </x:c>
+      <x:c r="B14" s="6" t="str">
+        <x:v>2026-10-24</x:v>
+      </x:c>
+      <x:c r="C14" s="2"/>
+      <x:c r="D14" s="2"/>
+      <x:c r="E14" s="2"/>
+      <x:c r="F14" s="2"/>
+    </x:row>
+    <x:row r="15" ht="24" customHeight="1">
+      <x:c r="A15" s="6" t="str">
+        <x:v>Reference source snapshot</x:v>
+      </x:c>
+      <x:c r="B15" s="6" t="str"/>
+      <x:c r="C15" s="2"/>
+      <x:c r="D15" s="2"/>
+      <x:c r="E15" s="2"/>
+      <x:c r="F15" s="2"/>
+    </x:row>
+    <x:row r="16" ht="65" customHeight="1">
+      <x:c r="A16" s="6" t="str">
+        <x:v>Scope</x:v>
+      </x:c>
+      <x:c r="B16" s="6" t="str">
+        <x:v>Optional: leave review flag 0 unless intentionally enabling a reviewed cash-funded recovery. Replace all six yearly operating-driver links with reviewed literal values in Driver Paths. Blank obligations are not zero. No new financing or dilution. Reimport after source or review changes.</x:v>
+      </x:c>
+      <x:c r="C16" s="2"/>
+      <x:c r="D16" s="2"/>
+      <x:c r="E16" s="2"/>
+      <x:c r="F16" s="2"/>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="40" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="23" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="23" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="23" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="23" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="23" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="24" customHeight="1">
+      <x:c r="A1" s="5" t="str">
+        <x:v>Driver / annual override</x:v>
+      </x:c>
+      <x:c r="B1" s="5" t="str">
+        <x:v>Y1</x:v>
+      </x:c>
+      <x:c r="C1" s="5" t="str">
+        <x:v>Y2</x:v>
+      </x:c>
+      <x:c r="D1" s="5" t="str">
+        <x:v>Y3</x:v>
+      </x:c>
+      <x:c r="E1" s="5" t="str">
+        <x:v>Y4</x:v>
+      </x:c>
+      <x:c r="F1" s="5" t="str">
+        <x:v>Y5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="24" customHeight="1">
+      <x:c r="A2" s="6" t="str">
+        <x:v>growth</x:v>
+      </x:c>
+      <x:c r="B2" s="12" t="n">
+        <x:f>Assumptions!B3</x:f>
+        <x:v>0.06</x:v>
+      </x:c>
+      <x:c r="C2" s="12" t="n">
+        <x:f>Assumptions!B3</x:f>
+        <x:v>0.06</x:v>
+      </x:c>
+      <x:c r="D2" s="12" t="n">
+        <x:f>Assumptions!B3</x:f>
+        <x:v>0.06</x:v>
+      </x:c>
+      <x:c r="E2" s="12" t="n">
+        <x:f>Assumptions!B3</x:f>
+        <x:v>0.06</x:v>
+      </x:c>
+      <x:c r="F2" s="12" t="n">
+        <x:f>Assumptions!B3</x:f>
+        <x:v>0.06</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="24" customHeight="1">
+      <x:c r="A3" s="6" t="str">
+        <x:v>margin</x:v>
+      </x:c>
+      <x:c r="B3" s="12" t="n">
+        <x:f>Assumptions!B4</x:f>
+        <x:v>0.25866666666666666</x:v>
+      </x:c>
+      <x:c r="C3" s="12" t="n">
+        <x:f>Assumptions!B4</x:f>
+        <x:v>0.25866666666666666</x:v>
+      </x:c>
+      <x:c r="D3" s="12" t="n">
+        <x:f>Assumptions!B4</x:f>
+        <x:v>0.25866666666666666</x:v>
+      </x:c>
+      <x:c r="E3" s="12" t="n">
+        <x:f>Assumptions!B4</x:f>
+        <x:v>0.25866666666666666</x:v>
+      </x:c>
+      <x:c r="F3" s="12" t="n">
+        <x:f>Assumptions!B4</x:f>
+        <x:v>0.25866666666666666</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="24" customHeight="1">
+      <x:c r="A4" s="6" t="str">
+        <x:v>tax</x:v>
+      </x:c>
+      <x:c r="B4" s="12" t="n">
+        <x:f>Assumptions!B5</x:f>
+        <x:v>0.22</x:v>
+      </x:c>
+      <x:c r="C4" s="12" t="n">
+        <x:f>Assumptions!B5</x:f>
+        <x:v>0.22</x:v>
+      </x:c>
+      <x:c r="D4" s="12" t="n">
+        <x:f>Assumptions!B5</x:f>
+        <x:v>0.22</x:v>
+      </x:c>
+      <x:c r="E4" s="12" t="n">
+        <x:f>Assumptions!B5</x:f>
+        <x:v>0.22</x:v>
+      </x:c>
+      <x:c r="F4" s="12" t="n">
+        <x:f>Assumptions!B5</x:f>
+        <x:v>0.22</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="24" customHeight="1">
+      <x:c r="A5" s="6" t="str">
+        <x:v>da</x:v>
+      </x:c>
+      <x:c r="B5" s="12" t="n">
+        <x:f>Assumptions!B6</x:f>
+        <x:v>0.19466666666666665</x:v>
+      </x:c>
+      <x:c r="C5" s="12" t="n">
+        <x:f>Assumptions!B6</x:f>
+        <x:v>0.19466666666666665</x:v>
+      </x:c>
+      <x:c r="D5" s="12" t="n">
+        <x:f>Assumptions!B6</x:f>
+        <x:v>0.19466666666666665</x:v>
+      </x:c>
+      <x:c r="E5" s="12" t="n">
+        <x:f>Assumptions!B6</x:f>
+        <x:v>0.19466666666666665</x:v>
+      </x:c>
+      <x:c r="F5" s="12" t="n">
+        <x:f>Assumptions!B6</x:f>
+        <x:v>0.19466666666666665</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="24" customHeight="1">
+      <x:c r="A6" s="6" t="str">
+        <x:v>capex</x:v>
+      </x:c>
+      <x:c r="B6" s="12" t="n">
+        <x:f>Assumptions!B7</x:f>
+        <x:v>0.055</x:v>
+      </x:c>
+      <x:c r="C6" s="12" t="n">
+        <x:f>Assumptions!B7</x:f>
+        <x:v>0.055</x:v>
+      </x:c>
+      <x:c r="D6" s="12" t="n">
+        <x:f>Assumptions!B7</x:f>
+        <x:v>0.055</x:v>
+      </x:c>
+      <x:c r="E6" s="12" t="n">
+        <x:f>Assumptions!B7</x:f>
+        <x:v>0.055</x:v>
+      </x:c>
+      <x:c r="F6" s="12" t="n">
+        <x:f>Assumptions!B7</x:f>
+        <x:v>0.055</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="24" customHeight="1">
+      <x:c r="A7" s="6" t="str">
+        <x:v>nwc</x:v>
+      </x:c>
+      <x:c r="B7" s="12" t="n">
+        <x:f>Assumptions!B8</x:f>
+        <x:v>0.04</x:v>
+      </x:c>
+      <x:c r="C7" s="12" t="n">
+        <x:f>Assumptions!B8</x:f>
+        <x:v>0.04</x:v>
+      </x:c>
+      <x:c r="D7" s="12" t="n">
+        <x:f>Assumptions!B8</x:f>
+        <x:v>0.04</x:v>
+      </x:c>
+      <x:c r="E7" s="12" t="n">
+        <x:f>Assumptions!B8</x:f>
+        <x:v>0.04</x:v>
+      </x:c>
+      <x:c r="F7" s="12" t="n">
+        <x:f>Assumptions!B8</x:f>
+        <x:v>0.04</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="24" customHeight="1">
+      <x:c r="A8" s="6" t="str">
+        <x:v>rf</x:v>
+      </x:c>
+      <x:c r="B8" s="12" t="n">
+        <x:f>Assumptions!B9</x:f>
+        <x:v>0.065</x:v>
+      </x:c>
+      <x:c r="C8" s="12" t="n">
+        <x:f>Assumptions!B9</x:f>
+        <x:v>0.065</x:v>
+      </x:c>
+      <x:c r="D8" s="12" t="n">
+        <x:f>Assumptions!B9</x:f>
+        <x:v>0.065</x:v>
+      </x:c>
+      <x:c r="E8" s="12" t="n">
+        <x:f>Assumptions!B9</x:f>
+        <x:v>0.065</x:v>
+      </x:c>
+      <x:c r="F8" s="12" t="n">
+        <x:f>Assumptions!B9</x:f>
+        <x:v>0.065</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="24" customHeight="1">
+      <x:c r="A9" s="6" t="str">
+        <x:v>beta</x:v>
+      </x:c>
+      <x:c r="B9" s="12" t="n">
+        <x:f>Assumptions!B10</x:f>
+        <x:v>0.9</x:v>
+      </x:c>
+      <x:c r="C9" s="12" t="n">
+        <x:f>Assumptions!B10</x:f>
+        <x:v>0.9</x:v>
+      </x:c>
+      <x:c r="D9" s="12" t="n">
+        <x:f>Assumptions!B10</x:f>
+        <x:v>0.9</x:v>
+      </x:c>
+      <x:c r="E9" s="12" t="n">
+        <x:f>Assumptions!B10</x:f>
+        <x:v>0.9</x:v>
+      </x:c>
+      <x:c r="F9" s="12" t="n">
+        <x:f>Assumptions!B10</x:f>
+        <x:v>0.9</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="24" customHeight="1">
+      <x:c r="A10" s="6" t="str">
+        <x:v>erp</x:v>
+      </x:c>
+      <x:c r="B10" s="12" t="n">
+        <x:f>Assumptions!B11</x:f>
+        <x:v>0.065</x:v>
+      </x:c>
+      <x:c r="C10" s="12" t="n">
+        <x:f>Assumptions!B11</x:f>
+        <x:v>0.065</x:v>
+      </x:c>
+      <x:c r="D10" s="12" t="n">
+        <x:f>Assumptions!B11</x:f>
+        <x:v>0.065</x:v>
+      </x:c>
+      <x:c r="E10" s="12" t="n">
+        <x:f>Assumptions!B11</x:f>
+        <x:v>0.065</x:v>
+      </x:c>
+      <x:c r="F10" s="12" t="n">
+        <x:f>Assumptions!B11</x:f>
+        <x:v>0.065</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="24" customHeight="1">
+      <x:c r="A11" s="6" t="str">
+        <x:v>kd</x:v>
+      </x:c>
+      <x:c r="B11" s="12" t="n">
+        <x:f>Assumptions!B12</x:f>
+        <x:v>0.085</x:v>
+      </x:c>
+      <x:c r="C11" s="12" t="n">
+        <x:f>Assumptions!B12</x:f>
+        <x:v>0.085</x:v>
+      </x:c>
+      <x:c r="D11" s="12" t="n">
+        <x:f>Assumptions!B12</x:f>
+        <x:v>0.085</x:v>
+      </x:c>
+      <x:c r="E11" s="12" t="n">
+        <x:f>Assumptions!B12</x:f>
+        <x:v>0.085</x:v>
+      </x:c>
+      <x:c r="F11" s="12" t="n">
+        <x:f>Assumptions!B12</x:f>
+        <x:v>0.085</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="24" customHeight="1">
+      <x:c r="A12" s="6" t="str">
+        <x:v>g</x:v>
+      </x:c>
+      <x:c r="B12" s="12" t="n">
+        <x:f>Assumptions!B13</x:f>
+        <x:v>0.035</x:v>
+      </x:c>
+      <x:c r="C12" s="12" t="n">
+        <x:f>Assumptions!B13</x:f>
+        <x:v>0.035</x:v>
+      </x:c>
+      <x:c r="D12" s="12" t="n">
+        <x:f>Assumptions!B13</x:f>
+        <x:v>0.035</x:v>
+      </x:c>
+      <x:c r="E12" s="12" t="n">
+        <x:f>Assumptions!B13</x:f>
+        <x:v>0.035</x:v>
+      </x:c>
+      <x:c r="F12" s="12" t="n">
+        <x:f>Assumptions!B13</x:f>
+        <x:v>0.035</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="24" customHeight="1">
+      <x:c r="A13" s="6" t="str">
+        <x:v>roic</x:v>
+      </x:c>
+      <x:c r="B13" s="12" t="n">
+        <x:f>Assumptions!B14</x:f>
+        <x:v>0.14</x:v>
+      </x:c>
+      <x:c r="C13" s="12" t="n">
+        <x:f>Assumptions!B14</x:f>
+        <x:v>0.14</x:v>
+      </x:c>
+      <x:c r="D13" s="12" t="n">
+        <x:f>Assumptions!B14</x:f>
+        <x:v>0.14</x:v>
+      </x:c>
+      <x:c r="E13" s="12" t="n">
+        <x:f>Assumptions!B14</x:f>
+        <x:v>0.14</x:v>
+      </x:c>
+      <x:c r="F13" s="12" t="n">
+        <x:f>Assumptions!B14</x:f>
+        <x:v>0.14</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="24" customHeight="1">
+      <x:c r="A14" s="6" t="str">
+        <x:v>payout</x:v>
+      </x:c>
+      <x:c r="B14" s="12" t="n">
+        <x:f>Assumptions!B15</x:f>
+        <x:v>0.65</x:v>
+      </x:c>
+      <x:c r="C14" s="12" t="n">
+        <x:f>Assumptions!B15</x:f>
+        <x:v>0.65</x:v>
+      </x:c>
+      <x:c r="D14" s="12" t="n">
+        <x:f>Assumptions!B15</x:f>
+        <x:v>0.65</x:v>
+      </x:c>
+      <x:c r="E14" s="12" t="n">
+        <x:f>Assumptions!B15</x:f>
+        <x:v>0.65</x:v>
+      </x:c>
+      <x:c r="F14" s="12" t="n">
+        <x:f>Assumptions!B15</x:f>
+        <x:v>0.65</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="24" customHeight="1">
+      <x:c r="A15" s="6" t="str">
+        <x:v>terminalRoe</x:v>
+      </x:c>
+      <x:c r="B15" s="12" t="n">
+        <x:f>Assumptions!B16</x:f>
+        <x:v>0.16</x:v>
+      </x:c>
+      <x:c r="C15" s="12" t="n">
+        <x:f>Assumptions!B16</x:f>
+        <x:v>0.16</x:v>
+      </x:c>
+      <x:c r="D15" s="12" t="n">
+        <x:f>Assumptions!B16</x:f>
+        <x:v>0.16</x:v>
+      </x:c>
+      <x:c r="E15" s="12" t="n">
+        <x:f>Assumptions!B16</x:f>
+        <x:v>0.16</x:v>
+      </x:c>
+      <x:c r="F15" s="12" t="n">
+        <x:f>Assumptions!B16</x:f>
+        <x:v>0.16</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="24" customHeight="1">
+      <x:c r="A16" s="6" t="str">
+        <x:v>buy</x:v>
+      </x:c>
+      <x:c r="B16" s="12" t="n">
+        <x:f>Assumptions!B17</x:f>
+        <x:v>0.15</x:v>
+      </x:c>
+      <x:c r="C16" s="12" t="n">
+        <x:f>Assumptions!B17</x:f>
+        <x:v>0.15</x:v>
+      </x:c>
+      <x:c r="D16" s="12" t="n">
+        <x:f>Assumptions!B17</x:f>
+        <x:v>0.15</x:v>
+      </x:c>
+      <x:c r="E16" s="12" t="n">
+        <x:f>Assumptions!B17</x:f>
+        <x:v>0.15</x:v>
+      </x:c>
+      <x:c r="F16" s="12" t="n">
+        <x:f>Assumptions!B17</x:f>
+        <x:v>0.15</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="24" customHeight="1">
+      <x:c r="A17" s="6" t="str">
+        <x:v>sell</x:v>
+      </x:c>
+      <x:c r="B17" s="12" t="n">
+        <x:f>Assumptions!B18</x:f>
+        <x:v>-0.15</x:v>
+      </x:c>
+      <x:c r="C17" s="12" t="n">
+        <x:f>Assumptions!B18</x:f>
+        <x:v>-0.15</x:v>
+      </x:c>
+      <x:c r="D17" s="12" t="n">
+        <x:f>Assumptions!B18</x:f>
+        <x:v>-0.15</x:v>
+      </x:c>
+      <x:c r="E17" s="12" t="n">
+        <x:f>Assumptions!B18</x:f>
+        <x:v>-0.15</x:v>
+      </x:c>
+      <x:c r="F17" s="12" t="n">
+        <x:f>Assumptions!B18</x:f>
+        <x:v>-0.15</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>